<commit_message>
Added a screenshot to the pricing tool to readme.md.
</commit_message>
<xml_diff>
--- a/notebooks/tools/used_car_pricing_tool.xlsx
+++ b/notebooks/tools/used_car_pricing_tool.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreylgoode/Documents/what-drives-car-prices/exports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreylgoode/Documents/what-drives-car-prices/notebooks/tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B877417D-06B6-2B47-B74C-21B9B9E007A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57776914-67FE-C440-A227-93606977507A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1780" windowWidth="28040" windowHeight="17440" xr2:uid="{1593D99B-1A1E-D64D-845E-99C9CF3821E3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Coefficients" sheetId="1" r:id="rId1"/>
-    <sheet name="Input" sheetId="2" r:id="rId2"/>
+    <sheet name="Input" sheetId="2" r:id="rId1"/>
+    <sheet name="Coefficients" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Coefficients!$A$1:$E$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Coefficients!$A$1:$E$70</definedName>
     <definedName name="collapsed_fuel">Coefficients!$N$7:$N$11</definedName>
     <definedName name="cylinders_list">Coefficients!$K$32:$K$35</definedName>
     <definedName name="drive_list">Coefficients!$L$39:$L$42</definedName>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="119">
   <si>
     <t>original_feature</t>
   </si>
@@ -393,10 +393,16 @@
     <t>Region</t>
   </si>
   <si>
-    <t>Manu Tier</t>
-  </si>
-  <si>
-    <t>Predicted Price</t>
+    <t>Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select Dropdown </t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Manufacturer Tier</t>
   </si>
 </sst>
 </file>
@@ -542,7 +548,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -722,8 +728,20 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -838,6 +856,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -883,10 +916,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1261,6 +1297,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{635B2F2D-52E1-0443-8331-B3F235E5BCEA}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="5">
+        <f>Coefficients!$E$1
++ _xlfn.XLOOKUP(B2, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B3, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B4, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B5, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B6, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B7, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B8, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B9, Coefficients!$B:$B, Coefficients!$C:$C)
++ _xlfn.XLOOKUP(B10, Coefficients!$B:$B, Coefficients!$C:$C)</f>
+        <v>15666.602150027931</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{30DA3E8D-90AF-8B4F-850D-2AA54BB330E2}">
+      <formula1>odometer_bins_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{D14D282F-699B-8643-8139-7DC89D0414B2}">
+      <formula1>year_bins_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4" xr:uid="{71A5A1DA-72F4-9343-B388-2F3A09C0F788}">
+      <formula1>type_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{8EA24209-5047-A94F-B620-5EEDA77739F4}">
+      <formula1>cylinders_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{ED74ADFD-77DA-BB42-9434-90649FA9CA03}">
+      <formula1>drive_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{DF231A89-6400-9D44-A968-3697857629E6}">
+      <formula1>transmission_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{579E8532-D534-EE46-A08B-A3CE1FB48D68}">
+      <formula1>collapsed_fuel</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9" xr:uid="{11E3E114-5113-3A4A-9E19-B0942E052E20}">
+      <formula1>region_list</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{DC50987D-5AD5-984C-8D24-C07D97485370}">
+      <formula1>Manufacturer_list</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE7C8DD-5BA4-944F-B298-A1596F202F13}">
   <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2255,137 +2432,4 @@
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{635B2F2D-52E1-0443-8331-B3F235E5BCEA}">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="17.5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>115</v>
-      </c>
-      <c r="B9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>116</v>
-      </c>
-      <c r="B11" s="2">
-        <f>Coefficients!$E$1
-+ _xlfn.XLOOKUP(B1, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B2, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B3, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B4, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B5, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B6, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B7, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B8, Coefficients!$B:$B, Coefficients!$C:$C)
-+ _xlfn.XLOOKUP(B9, Coefficients!$B:$B, Coefficients!$C:$C)</f>
-        <v>16242.242415183648</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="9">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1" xr:uid="{30DA3E8D-90AF-8B4F-850D-2AA54BB330E2}">
-      <formula1>odometer_bins_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{D14D282F-699B-8643-8139-7DC89D0414B2}">
-      <formula1>year_bins_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{71A5A1DA-72F4-9343-B388-2F3A09C0F788}">
-      <formula1>type_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4" xr:uid="{8EA24209-5047-A94F-B620-5EEDA77739F4}">
-      <formula1>cylinders_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{ED74ADFD-77DA-BB42-9434-90649FA9CA03}">
-      <formula1>drive_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{DF231A89-6400-9D44-A968-3697857629E6}">
-      <formula1>transmission_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{579E8532-D534-EE46-A08B-A3CE1FB48D68}">
-      <formula1>collapsed_fuel</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{11E3E114-5113-3A4A-9E19-B0942E052E20}">
-      <formula1>region_list</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9" xr:uid="{DC50987D-5AD5-984C-8D24-C07D97485370}">
-      <formula1>Manufacturer_list</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>